<commit_message>
control de errors hojas
</commit_message>
<xml_diff>
--- a/plantilla.xlsx
+++ b/plantilla.xlsx
@@ -8,20 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Desktop\clases\Carlos Excel\GBSOV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D3712A5-1D20-4304-8B47-BA6FF8FE1EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC1A46A8-1EE3-4435-B2E2-9CD3DFD209F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15345" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
     <sheet name="Mapping" sheetId="2" r:id="rId2"/>
-    <sheet name="BSC Data 02.2026" sheetId="3" r:id="rId3"/>
-    <sheet name="tabla dinamica mes anterior" sheetId="4" r:id="rId4"/>
-    <sheet name="BSC Data 01.2026" sheetId="5" r:id="rId5"/>
-    <sheet name="source" sheetId="6" r:id="rId6"/>
-    <sheet name="FDD " sheetId="7" r:id="rId7"/>
-    <sheet name="Reviewer" sheetId="8" r:id="rId8"/>
-    <sheet name="BSC Data 03.2026" sheetId="9" r:id="rId9"/>
+    <sheet name="tabla dinamica mes anterior" sheetId="4" r:id="rId3"/>
+    <sheet name="source" sheetId="6" r:id="rId4"/>
+    <sheet name="FDD " sheetId="7" r:id="rId5"/>
+    <sheet name="Reviewer" sheetId="8" r:id="rId6"/>
+    <sheet name="BSC Data 03.2026" sheetId="9" r:id="rId7"/>
+    <sheet name="BSC Data 04.2026" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -33,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="17">
   <si>
     <t>Invoice</t>
   </si>
@@ -59,16 +58,7 @@
     <t>dsfgsdfg</t>
   </si>
   <si>
-    <t xml:space="preserve">Ene </t>
-  </si>
-  <si>
     <t>Feb</t>
-  </si>
-  <si>
-    <t>mar</t>
-  </si>
-  <si>
-    <t>abr</t>
   </si>
   <si>
     <t>1. abrir archivo GBSOV hecho del ultimo mes</t>
@@ -521,93 +511,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F3792C0-B634-4537-AD97-15C4D5CE007E}">
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>6346</v>
-      </c>
-      <c r="B2">
-        <v>345634</v>
-      </c>
-      <c r="C2">
-        <v>768</v>
-      </c>
-      <c r="D2">
-        <v>9769</v>
-      </c>
-      <c r="E2">
-        <v>678967</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="I5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="I10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20135653-8DEC-40F8-A5DC-7908F893F36A}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -616,31 +519,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{780B7A86-CC9D-4A84-8C97-82F52135309D}">
-  <dimension ref="F2:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="2" spans="6:9" x14ac:dyDescent="0.25">
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24F1EC01-F583-4A00-8D2E-499FA316F2D8}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -649,7 +528,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{646D790B-EF2D-48A4-8EDA-71726D6B07B6}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -658,7 +537,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8AD4D87-03D9-4600-8D9C-B4EEB69A37A9}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -667,7 +546,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D37EF640-5235-45BD-ADD5-96914711108C}">
   <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -708,45 +587,132 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I9" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="I10" t="s">
-        <v>19</v>
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09FBB1C0-F95C-473C-9BAF-5FB60D7D5480}">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>6346</v>
+      </c>
+      <c r="B2">
+        <v>345634</v>
+      </c>
+      <c r="C2">
+        <v>768</v>
+      </c>
+      <c r="D2">
+        <v>9769</v>
+      </c>
+      <c r="E2">
+        <v>678967</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar con vlookup para obtener CC
</commit_message>
<xml_diff>
--- a/plantilla.xlsx
+++ b/plantilla.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6edcc1c4ba920e4e/Desktop/project/GBSOV/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{C5692DB7-1512-4192-B0E5-3461576DFEAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2033DEB8-33D2-4730-8AF9-97281EA7A644}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{C5692DB7-1512-4192-B0E5-3461576DFEAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F35A69B5-7B71-4C8E-90C6-0AC6104F7619}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" tabRatio="821" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="97">
   <si>
     <t>Invoice</t>
   </si>
@@ -280,6 +280,63 @@
   <si>
     <t>Grand Total</t>
   </si>
+  <si>
+    <t xml:space="preserve">Legal entity </t>
+  </si>
+  <si>
+    <t>External Id</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>GCRS</t>
+  </si>
+  <si>
+    <t>E605</t>
+  </si>
+  <si>
+    <t>TTREY</t>
+  </si>
+  <si>
+    <t>xxxxx</t>
+  </si>
+  <si>
+    <t>yyyyy</t>
+  </si>
+  <si>
+    <t>ERFC</t>
+  </si>
+  <si>
+    <t>TRGV</t>
+  </si>
+  <si>
+    <t>RECF</t>
+  </si>
+  <si>
+    <t>UUHY</t>
+  </si>
+  <si>
+    <t>HJLI</t>
+  </si>
+  <si>
+    <t>OIWE</t>
+  </si>
+  <si>
+    <t>GTFRE</t>
+  </si>
+  <si>
+    <t>DFCER</t>
+  </si>
+  <si>
+    <t>HHGVD</t>
+  </si>
+  <si>
+    <t>LOKKI</t>
+  </si>
+  <si>
+    <t>JUKHH</t>
+  </si>
 </sst>
 </file>
 
@@ -305,12 +362,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -340,12 +403,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -708,6 +772,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5762BC94-01DD-427A-8F95-7ABAD9B66525}">
   <dimension ref="A1:FE43"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="17" max="17" width="8.88671875" style="3"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:161" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -758,9 +825,6 @@
       <c r="P1" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" t="s">
-        <v>4</v>
-      </c>
       <c r="R1" t="s">
         <v>5</v>
       </c>
@@ -1079,7 +1143,7 @@
         <v>678967</v>
       </c>
       <c r="Q2">
-        <v>678967</v>
+        <v>39</v>
       </c>
       <c r="R2" t="s">
         <v>9</v>
@@ -1120,8 +1184,9 @@
       <c r="AD2">
         <v>678967</v>
       </c>
-      <c r="AE2" t="s">
-        <v>51</v>
+      <c r="AE2" s="3" t="str">
+        <f>VLOOKUP(Q2, Mapping!$D$2:$G$301,3,0)</f>
+        <v>ERFC</v>
       </c>
       <c r="AF2">
         <v>678967</v>
@@ -1512,7 +1577,7 @@
       </c>
       <c r="FE2" t="str">
         <f t="shared" ref="FE2:FE43" si="0">R2&amp;G2&amp;AE2</f>
-        <v>J6581234567899MMMM</v>
+        <v>J6581234567899ERFC</v>
       </c>
     </row>
     <row r="3" spans="1:161" x14ac:dyDescent="0.3">
@@ -1565,7 +1630,7 @@
         <v>678967</v>
       </c>
       <c r="Q3">
-        <v>678967</v>
+        <v>40</v>
       </c>
       <c r="R3" t="s">
         <v>10</v>
@@ -2051,7 +2116,7 @@
         <v>678967</v>
       </c>
       <c r="Q4">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R4" t="s">
         <v>11</v>
@@ -2537,7 +2602,7 @@
         <v>678967</v>
       </c>
       <c r="Q5">
-        <v>678967</v>
+        <v>125</v>
       </c>
       <c r="R5" t="s">
         <v>12</v>
@@ -3023,7 +3088,7 @@
         <v>678967</v>
       </c>
       <c r="Q6">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R6" t="s">
         <v>13</v>
@@ -3509,7 +3574,7 @@
         <v>678967</v>
       </c>
       <c r="Q7">
-        <v>678967</v>
+        <v>130</v>
       </c>
       <c r="R7" t="s">
         <v>14</v>
@@ -3995,7 +4060,7 @@
         <v>678967</v>
       </c>
       <c r="Q8">
-        <v>678967</v>
+        <v>39</v>
       </c>
       <c r="R8" t="s">
         <v>15</v>
@@ -4481,7 +4546,7 @@
         <v>678967</v>
       </c>
       <c r="Q9">
-        <v>678967</v>
+        <v>40</v>
       </c>
       <c r="R9" t="s">
         <v>16</v>
@@ -4967,7 +5032,7 @@
         <v>678967</v>
       </c>
       <c r="Q10">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R10" t="s">
         <v>17</v>
@@ -5453,7 +5518,7 @@
         <v>678967</v>
       </c>
       <c r="Q11">
-        <v>678967</v>
+        <v>125</v>
       </c>
       <c r="R11" t="s">
         <v>18</v>
@@ -5939,7 +6004,7 @@
         <v>678967</v>
       </c>
       <c r="Q12">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R12" t="s">
         <v>19</v>
@@ -6425,7 +6490,7 @@
         <v>678967</v>
       </c>
       <c r="Q13">
-        <v>678967</v>
+        <v>130</v>
       </c>
       <c r="R13" t="s">
         <v>20</v>
@@ -6911,7 +6976,7 @@
         <v>678967</v>
       </c>
       <c r="Q14">
-        <v>678967</v>
+        <v>39</v>
       </c>
       <c r="R14" t="s">
         <v>21</v>
@@ -7397,7 +7462,7 @@
         <v>678967</v>
       </c>
       <c r="Q15">
-        <v>678967</v>
+        <v>40</v>
       </c>
       <c r="R15" t="s">
         <v>22</v>
@@ -7883,7 +7948,7 @@
         <v>678967</v>
       </c>
       <c r="Q16">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R16" t="s">
         <v>23</v>
@@ -8369,7 +8434,7 @@
         <v>678967</v>
       </c>
       <c r="Q17">
-        <v>678967</v>
+        <v>125</v>
       </c>
       <c r="R17" t="s">
         <v>24</v>
@@ -8855,7 +8920,7 @@
         <v>678967</v>
       </c>
       <c r="Q18">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R18" t="s">
         <v>25</v>
@@ -9341,7 +9406,7 @@
         <v>678967</v>
       </c>
       <c r="Q19">
-        <v>678967</v>
+        <v>130</v>
       </c>
       <c r="R19" t="s">
         <v>26</v>
@@ -9826,7 +9891,7 @@
       <c r="P20">
         <v>678967</v>
       </c>
-      <c r="Q20">
+      <c r="Q20" s="3">
         <v>678967</v>
       </c>
       <c r="R20" t="s">
@@ -10312,7 +10377,7 @@
       <c r="P21">
         <v>678967</v>
       </c>
-      <c r="Q21">
+      <c r="Q21" s="3">
         <v>678967</v>
       </c>
       <c r="R21" t="s">
@@ -10798,7 +10863,7 @@
       <c r="P22">
         <v>678967</v>
       </c>
-      <c r="Q22">
+      <c r="Q22" s="3">
         <v>678967</v>
       </c>
       <c r="R22" t="s">
@@ -11284,7 +11349,7 @@
       <c r="P23">
         <v>678967</v>
       </c>
-      <c r="Q23">
+      <c r="Q23" s="3">
         <v>678967</v>
       </c>
       <c r="R23" t="s">
@@ -11770,7 +11835,7 @@
       <c r="P24">
         <v>678967</v>
       </c>
-      <c r="Q24">
+      <c r="Q24" s="3">
         <v>678967</v>
       </c>
       <c r="R24" t="s">
@@ -12256,7 +12321,7 @@
       <c r="P25">
         <v>678967</v>
       </c>
-      <c r="Q25">
+      <c r="Q25" s="3">
         <v>678967</v>
       </c>
       <c r="R25" t="s">
@@ -12742,7 +12807,7 @@
       <c r="P26">
         <v>678967</v>
       </c>
-      <c r="Q26">
+      <c r="Q26" s="3">
         <v>678967</v>
       </c>
       <c r="R26" t="s">
@@ -13228,7 +13293,7 @@
       <c r="P27">
         <v>678967</v>
       </c>
-      <c r="Q27">
+      <c r="Q27" s="3">
         <v>678967</v>
       </c>
       <c r="R27" t="s">
@@ -13714,7 +13779,7 @@
       <c r="P28">
         <v>678967</v>
       </c>
-      <c r="Q28">
+      <c r="Q28" s="3">
         <v>678967</v>
       </c>
       <c r="R28" t="s">
@@ -14200,7 +14265,7 @@
       <c r="P29">
         <v>678967</v>
       </c>
-      <c r="Q29">
+      <c r="Q29" s="3">
         <v>678967</v>
       </c>
       <c r="R29" t="s">
@@ -14686,7 +14751,7 @@
       <c r="P30">
         <v>678967</v>
       </c>
-      <c r="Q30">
+      <c r="Q30" s="3">
         <v>678967</v>
       </c>
       <c r="R30" t="s">
@@ -15172,7 +15237,7 @@
       <c r="P31">
         <v>678967</v>
       </c>
-      <c r="Q31">
+      <c r="Q31" s="3">
         <v>678967</v>
       </c>
       <c r="R31" t="s">
@@ -15658,7 +15723,7 @@
       <c r="P32">
         <v>678967</v>
       </c>
-      <c r="Q32">
+      <c r="Q32" s="3">
         <v>678967</v>
       </c>
       <c r="R32" t="s">
@@ -16144,7 +16209,7 @@
       <c r="P33">
         <v>678967</v>
       </c>
-      <c r="Q33">
+      <c r="Q33" s="3">
         <v>678967</v>
       </c>
       <c r="R33" t="s">
@@ -16630,7 +16695,7 @@
       <c r="P34">
         <v>678967</v>
       </c>
-      <c r="Q34">
+      <c r="Q34" s="3">
         <v>678967</v>
       </c>
       <c r="R34" t="s">
@@ -17116,7 +17181,7 @@
       <c r="P35">
         <v>678967</v>
       </c>
-      <c r="Q35">
+      <c r="Q35" s="3">
         <v>678967</v>
       </c>
       <c r="R35" t="s">
@@ -17602,7 +17667,7 @@
       <c r="P36">
         <v>678967</v>
       </c>
-      <c r="Q36">
+      <c r="Q36" s="3">
         <v>678967</v>
       </c>
       <c r="R36" t="s">
@@ -18088,7 +18153,7 @@
       <c r="P37">
         <v>678967</v>
       </c>
-      <c r="Q37">
+      <c r="Q37" s="3">
         <v>678967</v>
       </c>
       <c r="R37" t="s">
@@ -18574,7 +18639,7 @@
       <c r="P38">
         <v>678967</v>
       </c>
-      <c r="Q38">
+      <c r="Q38" s="3">
         <v>678967</v>
       </c>
       <c r="R38" t="s">
@@ -19060,7 +19125,7 @@
       <c r="P39">
         <v>678967</v>
       </c>
-      <c r="Q39">
+      <c r="Q39" s="3">
         <v>678967</v>
       </c>
       <c r="R39" t="s">
@@ -19546,7 +19611,7 @@
       <c r="P40">
         <v>678967</v>
       </c>
-      <c r="Q40">
+      <c r="Q40" s="3">
         <v>678967</v>
       </c>
       <c r="R40" t="s">
@@ -20032,7 +20097,7 @@
       <c r="P41">
         <v>678967</v>
       </c>
-      <c r="Q41">
+      <c r="Q41" s="3">
         <v>678967</v>
       </c>
       <c r="R41" t="s">
@@ -20518,7 +20583,7 @@
       <c r="P42">
         <v>678967</v>
       </c>
-      <c r="Q42">
+      <c r="Q42" s="3">
         <v>678967</v>
       </c>
       <c r="R42" t="s">
@@ -21004,7 +21069,7 @@
       <c r="P43">
         <v>678967</v>
       </c>
-      <c r="Q43">
+      <c r="Q43" s="3">
         <v>678967</v>
       </c>
       <c r="R43" t="s">
@@ -21448,9 +21513,203 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA7C9B72-FB0C-44D3-A18B-A9F10242A995}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G2" t="s">
+        <v>85</v>
+      </c>
+      <c r="H2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4">
+        <v>105</v>
+      </c>
+      <c r="E4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>88</v>
+      </c>
+      <c r="G4" t="s">
+        <v>85</v>
+      </c>
+      <c r="H4">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D5">
+        <v>125</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H5">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6">
+        <v>105</v>
+      </c>
+      <c r="E6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" t="s">
+        <v>90</v>
+      </c>
+      <c r="G6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H6">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7">
+        <v>130</v>
+      </c>
+      <c r="E7" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" t="s">
+        <v>85</v>
+      </c>
+      <c r="H7">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -61708,6 +61967,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.88671875" style="3"/>
     <col min="161" max="161" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -61778,7 +62038,7 @@
         <v>678967</v>
       </c>
       <c r="Q2">
-        <v>678967</v>
+        <v>39</v>
       </c>
       <c r="R2" t="s">
         <v>9</v>
@@ -61819,8 +62079,9 @@
       <c r="AD2">
         <v>678967</v>
       </c>
-      <c r="AE2" t="s">
-        <v>51</v>
+      <c r="AE2" s="3" t="str">
+        <f>VLOOKUP(Q2, Mapping!$D$2:$G$301,3,0)</f>
+        <v>ERFC</v>
       </c>
       <c r="AF2">
         <v>678967</v>
@@ -62211,7 +62472,7 @@
       </c>
       <c r="FE2" t="str">
         <f t="shared" ref="FE2:FE43" si="0">R2&amp;G2&amp;AE2</f>
-        <v>J6581234567899MMMM</v>
+        <v>J6581234567899ERFC</v>
       </c>
     </row>
     <row r="3" spans="1:161" x14ac:dyDescent="0.3">
@@ -62264,7 +62525,7 @@
         <v>678967</v>
       </c>
       <c r="Q3">
-        <v>678967</v>
+        <v>40</v>
       </c>
       <c r="R3" t="s">
         <v>10</v>
@@ -62305,8 +62566,9 @@
       <c r="AD3">
         <v>678967</v>
       </c>
-      <c r="AE3" t="s">
-        <v>51</v>
+      <c r="AE3" t="str">
+        <f>VLOOKUP(Q3, Mapping!$D$2:$G$301,3,0)</f>
+        <v>TRGV</v>
       </c>
       <c r="AF3">
         <v>678967</v>
@@ -62697,7 +62959,7 @@
       </c>
       <c r="FE3" t="str">
         <f t="shared" si="0"/>
-        <v>J659123456789MMMM</v>
+        <v>J659123456789TRGV</v>
       </c>
     </row>
     <row r="4" spans="1:161" x14ac:dyDescent="0.3">
@@ -62750,7 +63012,7 @@
         <v>678967</v>
       </c>
       <c r="Q4">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R4" t="s">
         <v>11</v>
@@ -62791,8 +63053,9 @@
       <c r="AD4">
         <v>678967</v>
       </c>
-      <c r="AE4" t="s">
-        <v>51</v>
+      <c r="AE4" t="str">
+        <f>VLOOKUP(Q4, Mapping!$D$2:$G$301,3,0)</f>
+        <v>RECF</v>
       </c>
       <c r="AF4">
         <v>678967</v>
@@ -63183,7 +63446,7 @@
       </c>
       <c r="FE4" t="str">
         <f t="shared" si="0"/>
-        <v>J660123456789MMMM</v>
+        <v>J660123456789RECF</v>
       </c>
     </row>
     <row r="5" spans="1:161" x14ac:dyDescent="0.3">
@@ -63236,7 +63499,7 @@
         <v>678967</v>
       </c>
       <c r="Q5">
-        <v>678967</v>
+        <v>125</v>
       </c>
       <c r="R5" t="s">
         <v>12</v>
@@ -63277,8 +63540,9 @@
       <c r="AD5">
         <v>678967</v>
       </c>
-      <c r="AE5" t="s">
-        <v>51</v>
+      <c r="AE5" t="str">
+        <f>VLOOKUP(Q5, Mapping!$D$2:$G$301,3,0)</f>
+        <v>UUHY</v>
       </c>
       <c r="AF5">
         <v>678967</v>
@@ -63669,7 +63933,7 @@
       </c>
       <c r="FE5" t="str">
         <f t="shared" si="0"/>
-        <v>J661123456789MMMM</v>
+        <v>J661123456789UUHY</v>
       </c>
     </row>
     <row r="6" spans="1:161" x14ac:dyDescent="0.3">
@@ -63722,7 +63986,7 @@
         <v>678967</v>
       </c>
       <c r="Q6">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R6" t="s">
         <v>13</v>
@@ -63763,8 +64027,9 @@
       <c r="AD6">
         <v>678967</v>
       </c>
-      <c r="AE6" t="s">
-        <v>51</v>
+      <c r="AE6" t="str">
+        <f>VLOOKUP(Q6, Mapping!$D$2:$G$301,3,0)</f>
+        <v>RECF</v>
       </c>
       <c r="AF6">
         <v>678967</v>
@@ -64155,7 +64420,7 @@
       </c>
       <c r="FE6" t="str">
         <f t="shared" si="0"/>
-        <v>J662123456789MMMM</v>
+        <v>J662123456789RECF</v>
       </c>
     </row>
     <row r="7" spans="1:161" x14ac:dyDescent="0.3">
@@ -64208,7 +64473,7 @@
         <v>678967</v>
       </c>
       <c r="Q7">
-        <v>678967</v>
+        <v>130</v>
       </c>
       <c r="R7" t="s">
         <v>14</v>
@@ -64249,8 +64514,9 @@
       <c r="AD7">
         <v>678967</v>
       </c>
-      <c r="AE7" t="s">
-        <v>51</v>
+      <c r="AE7" t="str">
+        <f>VLOOKUP(Q7, Mapping!$D$2:$G$301,3,0)</f>
+        <v>OIWE</v>
       </c>
       <c r="AF7">
         <v>678967</v>
@@ -64641,7 +64907,7 @@
       </c>
       <c r="FE7" t="str">
         <f t="shared" si="0"/>
-        <v>J663123456789MMMM</v>
+        <v>J663123456789OIWE</v>
       </c>
     </row>
     <row r="8" spans="1:161" x14ac:dyDescent="0.3">
@@ -64694,7 +64960,7 @@
         <v>678967</v>
       </c>
       <c r="Q8">
-        <v>678967</v>
+        <v>39</v>
       </c>
       <c r="R8" t="s">
         <v>15</v>
@@ -64735,8 +65001,9 @@
       <c r="AD8">
         <v>678967</v>
       </c>
-      <c r="AE8" t="s">
-        <v>51</v>
+      <c r="AE8" t="str">
+        <f>VLOOKUP(Q8, Mapping!$D$2:$G$301,3,0)</f>
+        <v>ERFC</v>
       </c>
       <c r="AF8">
         <v>678967</v>
@@ -65127,7 +65394,7 @@
       </c>
       <c r="FE8" t="str">
         <f t="shared" si="0"/>
-        <v>J664123456789MMMM</v>
+        <v>J664123456789ERFC</v>
       </c>
     </row>
     <row r="9" spans="1:161" x14ac:dyDescent="0.3">
@@ -65180,7 +65447,7 @@
         <v>678967</v>
       </c>
       <c r="Q9">
-        <v>678967</v>
+        <v>40</v>
       </c>
       <c r="R9" t="s">
         <v>16</v>
@@ -65221,8 +65488,9 @@
       <c r="AD9">
         <v>678967</v>
       </c>
-      <c r="AE9" t="s">
-        <v>51</v>
+      <c r="AE9" t="str">
+        <f>VLOOKUP(Q9, Mapping!$D$2:$G$301,3,0)</f>
+        <v>TRGV</v>
       </c>
       <c r="AF9">
         <v>678967</v>
@@ -65613,7 +65881,7 @@
       </c>
       <c r="FE9" t="str">
         <f t="shared" si="0"/>
-        <v>J665123456789MMMM</v>
+        <v>J665123456789TRGV</v>
       </c>
     </row>
     <row r="10" spans="1:161" x14ac:dyDescent="0.3">
@@ -65666,7 +65934,7 @@
         <v>678967</v>
       </c>
       <c r="Q10">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R10" t="s">
         <v>17</v>
@@ -65707,8 +65975,9 @@
       <c r="AD10">
         <v>678967</v>
       </c>
-      <c r="AE10" t="s">
-        <v>51</v>
+      <c r="AE10" t="str">
+        <f>VLOOKUP(Q10, Mapping!$D$2:$G$301,3,0)</f>
+        <v>RECF</v>
       </c>
       <c r="AF10">
         <v>678967</v>
@@ -66099,7 +66368,7 @@
       </c>
       <c r="FE10" t="str">
         <f t="shared" si="0"/>
-        <v>J666123456789MMMM</v>
+        <v>J666123456789RECF</v>
       </c>
     </row>
     <row r="11" spans="1:161" x14ac:dyDescent="0.3">
@@ -66152,7 +66421,7 @@
         <v>678967</v>
       </c>
       <c r="Q11">
-        <v>678967</v>
+        <v>125</v>
       </c>
       <c r="R11" t="s">
         <v>18</v>
@@ -66193,8 +66462,9 @@
       <c r="AD11">
         <v>678967</v>
       </c>
-      <c r="AE11" t="s">
-        <v>51</v>
+      <c r="AE11" t="str">
+        <f>VLOOKUP(Q11, Mapping!$D$2:$G$301,3,0)</f>
+        <v>UUHY</v>
       </c>
       <c r="AF11">
         <v>678967</v>
@@ -66585,7 +66855,7 @@
       </c>
       <c r="FE11" t="str">
         <f t="shared" si="0"/>
-        <v>J667123456789MMMM</v>
+        <v>J667123456789UUHY</v>
       </c>
     </row>
     <row r="12" spans="1:161" x14ac:dyDescent="0.3">
@@ -66638,7 +66908,7 @@
         <v>678967</v>
       </c>
       <c r="Q12">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R12" t="s">
         <v>19</v>
@@ -66679,8 +66949,9 @@
       <c r="AD12">
         <v>678967</v>
       </c>
-      <c r="AE12" t="s">
-        <v>51</v>
+      <c r="AE12" t="str">
+        <f>VLOOKUP(Q12, Mapping!$D$2:$G$301,3,0)</f>
+        <v>RECF</v>
       </c>
       <c r="AF12">
         <v>678967</v>
@@ -67071,7 +67342,7 @@
       </c>
       <c r="FE12" t="str">
         <f t="shared" si="0"/>
-        <v>J668123456789MMMM</v>
+        <v>J668123456789RECF</v>
       </c>
     </row>
     <row r="13" spans="1:161" x14ac:dyDescent="0.3">
@@ -67124,7 +67395,7 @@
         <v>678967</v>
       </c>
       <c r="Q13">
-        <v>678967</v>
+        <v>130</v>
       </c>
       <c r="R13" t="s">
         <v>20</v>
@@ -67165,8 +67436,9 @@
       <c r="AD13">
         <v>678967</v>
       </c>
-      <c r="AE13" t="s">
-        <v>51</v>
+      <c r="AE13" t="str">
+        <f>VLOOKUP(Q13, Mapping!$D$2:$G$301,3,0)</f>
+        <v>OIWE</v>
       </c>
       <c r="AF13">
         <v>678967</v>
@@ -67557,7 +67829,7 @@
       </c>
       <c r="FE13" t="str">
         <f t="shared" si="0"/>
-        <v>J669123456789MMMM</v>
+        <v>J669123456789OIWE</v>
       </c>
     </row>
     <row r="14" spans="1:161" x14ac:dyDescent="0.3">
@@ -67610,7 +67882,7 @@
         <v>678967</v>
       </c>
       <c r="Q14">
-        <v>678967</v>
+        <v>39</v>
       </c>
       <c r="R14" t="s">
         <v>21</v>
@@ -67651,8 +67923,9 @@
       <c r="AD14">
         <v>678967</v>
       </c>
-      <c r="AE14" t="s">
-        <v>51</v>
+      <c r="AE14" t="str">
+        <f>VLOOKUP(Q14, Mapping!$D$2:$G$301,3,0)</f>
+        <v>ERFC</v>
       </c>
       <c r="AF14">
         <v>678967</v>
@@ -68043,7 +68316,7 @@
       </c>
       <c r="FE14" t="str">
         <f t="shared" si="0"/>
-        <v>J670123456789MMMM</v>
+        <v>J670123456789ERFC</v>
       </c>
     </row>
     <row r="15" spans="1:161" x14ac:dyDescent="0.3">
@@ -68096,7 +68369,7 @@
         <v>678967</v>
       </c>
       <c r="Q15">
-        <v>678967</v>
+        <v>40</v>
       </c>
       <c r="R15" t="s">
         <v>22</v>
@@ -68137,8 +68410,9 @@
       <c r="AD15">
         <v>678967</v>
       </c>
-      <c r="AE15" t="s">
-        <v>51</v>
+      <c r="AE15" t="str">
+        <f>VLOOKUP(Q15, Mapping!$D$2:$G$301,3,0)</f>
+        <v>TRGV</v>
       </c>
       <c r="AF15">
         <v>678967</v>
@@ -68529,7 +68803,7 @@
       </c>
       <c r="FE15" t="str">
         <f t="shared" si="0"/>
-        <v>J671123456789MMMM</v>
+        <v>J671123456789TRGV</v>
       </c>
     </row>
     <row r="16" spans="1:161" x14ac:dyDescent="0.3">
@@ -68582,7 +68856,7 @@
         <v>678967</v>
       </c>
       <c r="Q16">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R16" t="s">
         <v>23</v>
@@ -68623,8 +68897,9 @@
       <c r="AD16">
         <v>678967</v>
       </c>
-      <c r="AE16" t="s">
-        <v>51</v>
+      <c r="AE16" t="str">
+        <f>VLOOKUP(Q16, Mapping!$D$2:$G$301,3,0)</f>
+        <v>RECF</v>
       </c>
       <c r="AF16">
         <v>678967</v>
@@ -69015,7 +69290,7 @@
       </c>
       <c r="FE16" t="str">
         <f t="shared" si="0"/>
-        <v>J672123456789MMMM</v>
+        <v>J672123456789RECF</v>
       </c>
     </row>
     <row r="17" spans="1:161" x14ac:dyDescent="0.3">
@@ -69068,7 +69343,7 @@
         <v>678967</v>
       </c>
       <c r="Q17">
-        <v>678967</v>
+        <v>125</v>
       </c>
       <c r="R17" t="s">
         <v>24</v>
@@ -69109,8 +69384,9 @@
       <c r="AD17">
         <v>678967</v>
       </c>
-      <c r="AE17" t="s">
-        <v>51</v>
+      <c r="AE17" t="str">
+        <f>VLOOKUP(Q17, Mapping!$D$2:$G$301,3,0)</f>
+        <v>UUHY</v>
       </c>
       <c r="AF17">
         <v>678967</v>
@@ -69501,7 +69777,7 @@
       </c>
       <c r="FE17" t="str">
         <f t="shared" si="0"/>
-        <v>J673123456789MMMM</v>
+        <v>J673123456789UUHY</v>
       </c>
     </row>
     <row r="18" spans="1:161" x14ac:dyDescent="0.3">
@@ -69554,7 +69830,7 @@
         <v>678967</v>
       </c>
       <c r="Q18">
-        <v>678967</v>
+        <v>105</v>
       </c>
       <c r="R18" t="s">
         <v>25</v>
@@ -69595,8 +69871,9 @@
       <c r="AD18">
         <v>678967</v>
       </c>
-      <c r="AE18" t="s">
-        <v>51</v>
+      <c r="AE18" t="str">
+        <f>VLOOKUP(Q18, Mapping!$D$2:$G$301,3,0)</f>
+        <v>RECF</v>
       </c>
       <c r="AF18">
         <v>678967</v>
@@ -69987,7 +70264,7 @@
       </c>
       <c r="FE18" t="str">
         <f t="shared" si="0"/>
-        <v>J674123456789MMMM</v>
+        <v>J674123456789RECF</v>
       </c>
     </row>
     <row r="19" spans="1:161" x14ac:dyDescent="0.3">
@@ -70040,7 +70317,7 @@
         <v>678967</v>
       </c>
       <c r="Q19">
-        <v>678967</v>
+        <v>130</v>
       </c>
       <c r="R19" t="s">
         <v>26</v>
@@ -70081,8 +70358,9 @@
       <c r="AD19">
         <v>678967</v>
       </c>
-      <c r="AE19" t="s">
-        <v>51</v>
+      <c r="AE19" t="str">
+        <f>VLOOKUP(Q19, Mapping!$D$2:$G$301,3,0)</f>
+        <v>OIWE</v>
       </c>
       <c r="AF19">
         <v>678967</v>
@@ -70473,7 +70751,7 @@
       </c>
       <c r="FE19" t="str">
         <f t="shared" si="0"/>
-        <v>J675123456789MMMM</v>
+        <v>J675123456789OIWE</v>
       </c>
     </row>
     <row r="20" spans="1:161" x14ac:dyDescent="0.3">
@@ -70525,7 +70803,7 @@
       <c r="P20">
         <v>678967</v>
       </c>
-      <c r="Q20">
+      <c r="Q20" s="3">
         <v>678967</v>
       </c>
       <c r="R20" t="s">
@@ -70567,8 +70845,9 @@
       <c r="AD20">
         <v>678967</v>
       </c>
-      <c r="AE20" t="s">
-        <v>51</v>
+      <c r="AE20" t="e">
+        <f>VLOOKUP(Q20, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF20">
         <v>678967</v>
@@ -70957,9 +71236,9 @@
       <c r="FD20">
         <v>678967</v>
       </c>
-      <c r="FE20" t="str">
+      <c r="FE20" t="e">
         <f t="shared" si="0"/>
-        <v>J676123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="21" spans="1:161" x14ac:dyDescent="0.3">
@@ -71011,7 +71290,7 @@
       <c r="P21">
         <v>678967</v>
       </c>
-      <c r="Q21">
+      <c r="Q21" s="3">
         <v>678967</v>
       </c>
       <c r="R21" t="s">
@@ -71053,8 +71332,9 @@
       <c r="AD21">
         <v>678967</v>
       </c>
-      <c r="AE21" t="s">
-        <v>51</v>
+      <c r="AE21" t="e">
+        <f>VLOOKUP(Q21, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF21">
         <v>678967</v>
@@ -71443,9 +71723,9 @@
       <c r="FD21">
         <v>678967</v>
       </c>
-      <c r="FE21" t="str">
+      <c r="FE21" t="e">
         <f t="shared" si="0"/>
-        <v>J677123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="22" spans="1:161" x14ac:dyDescent="0.3">
@@ -71497,7 +71777,7 @@
       <c r="P22">
         <v>678967</v>
       </c>
-      <c r="Q22">
+      <c r="Q22" s="3">
         <v>678967</v>
       </c>
       <c r="R22" t="s">
@@ -71539,8 +71819,9 @@
       <c r="AD22">
         <v>678967</v>
       </c>
-      <c r="AE22" t="s">
-        <v>51</v>
+      <c r="AE22" t="e">
+        <f>VLOOKUP(Q22, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF22">
         <v>678967</v>
@@ -71929,9 +72210,9 @@
       <c r="FD22">
         <v>678967</v>
       </c>
-      <c r="FE22" t="str">
+      <c r="FE22" t="e">
         <f t="shared" si="0"/>
-        <v>J678123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="23" spans="1:161" x14ac:dyDescent="0.3">
@@ -71983,7 +72264,7 @@
       <c r="P23">
         <v>678967</v>
       </c>
-      <c r="Q23">
+      <c r="Q23" s="3">
         <v>678967</v>
       </c>
       <c r="R23" t="s">
@@ -72025,8 +72306,9 @@
       <c r="AD23">
         <v>678967</v>
       </c>
-      <c r="AE23" t="s">
-        <v>51</v>
+      <c r="AE23" t="e">
+        <f>VLOOKUP(Q23, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF23">
         <v>678967</v>
@@ -72415,9 +72697,9 @@
       <c r="FD23">
         <v>678967</v>
       </c>
-      <c r="FE23" t="str">
+      <c r="FE23" t="e">
         <f t="shared" si="0"/>
-        <v>J679123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="24" spans="1:161" x14ac:dyDescent="0.3">
@@ -72469,7 +72751,7 @@
       <c r="P24">
         <v>678967</v>
       </c>
-      <c r="Q24">
+      <c r="Q24" s="3">
         <v>678967</v>
       </c>
       <c r="R24" t="s">
@@ -72511,8 +72793,9 @@
       <c r="AD24">
         <v>678967</v>
       </c>
-      <c r="AE24" t="s">
-        <v>51</v>
+      <c r="AE24" t="e">
+        <f>VLOOKUP(Q24, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF24">
         <v>678967</v>
@@ -72901,9 +73184,9 @@
       <c r="FD24">
         <v>678967</v>
       </c>
-      <c r="FE24" t="str">
+      <c r="FE24" t="e">
         <f t="shared" si="0"/>
-        <v>J680123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="25" spans="1:161" x14ac:dyDescent="0.3">
@@ -72955,7 +73238,7 @@
       <c r="P25">
         <v>678967</v>
       </c>
-      <c r="Q25">
+      <c r="Q25" s="3">
         <v>678967</v>
       </c>
       <c r="R25" t="s">
@@ -72997,8 +73280,9 @@
       <c r="AD25">
         <v>678967</v>
       </c>
-      <c r="AE25" t="s">
-        <v>51</v>
+      <c r="AE25" t="e">
+        <f>VLOOKUP(Q25, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF25">
         <v>678967</v>
@@ -73387,9 +73671,9 @@
       <c r="FD25">
         <v>678967</v>
       </c>
-      <c r="FE25" t="str">
+      <c r="FE25" t="e">
         <f t="shared" si="0"/>
-        <v>J681123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="26" spans="1:161" x14ac:dyDescent="0.3">
@@ -73441,7 +73725,7 @@
       <c r="P26">
         <v>678967</v>
       </c>
-      <c r="Q26">
+      <c r="Q26" s="3">
         <v>678967</v>
       </c>
       <c r="R26" t="s">
@@ -73483,8 +73767,9 @@
       <c r="AD26">
         <v>678967</v>
       </c>
-      <c r="AE26" t="s">
-        <v>51</v>
+      <c r="AE26" t="e">
+        <f>VLOOKUP(Q26, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF26">
         <v>678967</v>
@@ -73873,9 +74158,9 @@
       <c r="FD26">
         <v>678967</v>
       </c>
-      <c r="FE26" t="str">
+      <c r="FE26" t="e">
         <f t="shared" si="0"/>
-        <v>J682123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="27" spans="1:161" x14ac:dyDescent="0.3">
@@ -73927,7 +74212,7 @@
       <c r="P27">
         <v>678967</v>
       </c>
-      <c r="Q27">
+      <c r="Q27" s="3">
         <v>678967</v>
       </c>
       <c r="R27" t="s">
@@ -73969,8 +74254,9 @@
       <c r="AD27">
         <v>678967</v>
       </c>
-      <c r="AE27" t="s">
-        <v>51</v>
+      <c r="AE27" t="e">
+        <f>VLOOKUP(Q27, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF27">
         <v>678967</v>
@@ -74359,9 +74645,9 @@
       <c r="FD27">
         <v>678967</v>
       </c>
-      <c r="FE27" t="str">
+      <c r="FE27" t="e">
         <f t="shared" si="0"/>
-        <v>J683123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="28" spans="1:161" x14ac:dyDescent="0.3">
@@ -74413,7 +74699,7 @@
       <c r="P28">
         <v>678967</v>
       </c>
-      <c r="Q28">
+      <c r="Q28" s="3">
         <v>678967</v>
       </c>
       <c r="R28" t="s">
@@ -74455,8 +74741,9 @@
       <c r="AD28">
         <v>678967</v>
       </c>
-      <c r="AE28" t="s">
-        <v>51</v>
+      <c r="AE28" t="e">
+        <f>VLOOKUP(Q28, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF28">
         <v>678967</v>
@@ -74845,9 +75132,9 @@
       <c r="FD28">
         <v>678967</v>
       </c>
-      <c r="FE28" t="str">
+      <c r="FE28" t="e">
         <f t="shared" si="0"/>
-        <v>J684123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="29" spans="1:161" x14ac:dyDescent="0.3">
@@ -74899,7 +75186,7 @@
       <c r="P29">
         <v>678967</v>
       </c>
-      <c r="Q29">
+      <c r="Q29" s="3">
         <v>678967</v>
       </c>
       <c r="R29" t="s">
@@ -74941,8 +75228,9 @@
       <c r="AD29">
         <v>678967</v>
       </c>
-      <c r="AE29" t="s">
-        <v>51</v>
+      <c r="AE29" t="e">
+        <f>VLOOKUP(Q29, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF29">
         <v>678967</v>
@@ -75331,9 +75619,9 @@
       <c r="FD29">
         <v>678967</v>
       </c>
-      <c r="FE29" t="str">
+      <c r="FE29" t="e">
         <f t="shared" si="0"/>
-        <v>J685123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="30" spans="1:161" x14ac:dyDescent="0.3">
@@ -75385,7 +75673,7 @@
       <c r="P30">
         <v>678967</v>
       </c>
-      <c r="Q30">
+      <c r="Q30" s="3">
         <v>678967</v>
       </c>
       <c r="R30" t="s">
@@ -75427,8 +75715,9 @@
       <c r="AD30">
         <v>678967</v>
       </c>
-      <c r="AE30" t="s">
-        <v>51</v>
+      <c r="AE30" t="e">
+        <f>VLOOKUP(Q30, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF30">
         <v>678967</v>
@@ -75817,9 +76106,9 @@
       <c r="FD30">
         <v>678967</v>
       </c>
-      <c r="FE30" t="str">
+      <c r="FE30" t="e">
         <f t="shared" si="0"/>
-        <v>J686123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="31" spans="1:161" x14ac:dyDescent="0.3">
@@ -75871,7 +76160,7 @@
       <c r="P31">
         <v>678967</v>
       </c>
-      <c r="Q31">
+      <c r="Q31" s="3">
         <v>678967</v>
       </c>
       <c r="R31" t="s">
@@ -75913,8 +76202,9 @@
       <c r="AD31">
         <v>678967</v>
       </c>
-      <c r="AE31" t="s">
-        <v>51</v>
+      <c r="AE31" t="e">
+        <f>VLOOKUP(Q31, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF31">
         <v>678967</v>
@@ -76303,9 +76593,9 @@
       <c r="FD31">
         <v>678967</v>
       </c>
-      <c r="FE31" t="str">
+      <c r="FE31" t="e">
         <f t="shared" si="0"/>
-        <v>J687123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="32" spans="1:161" x14ac:dyDescent="0.3">
@@ -76357,7 +76647,7 @@
       <c r="P32">
         <v>678967</v>
       </c>
-      <c r="Q32">
+      <c r="Q32" s="3">
         <v>678967</v>
       </c>
       <c r="R32" t="s">
@@ -76399,8 +76689,9 @@
       <c r="AD32">
         <v>678967</v>
       </c>
-      <c r="AE32" t="s">
-        <v>51</v>
+      <c r="AE32" t="e">
+        <f>VLOOKUP(Q32, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF32">
         <v>678967</v>
@@ -76789,9 +77080,9 @@
       <c r="FD32">
         <v>678967</v>
       </c>
-      <c r="FE32" t="str">
+      <c r="FE32" t="e">
         <f t="shared" si="0"/>
-        <v>J688123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="33" spans="1:161" x14ac:dyDescent="0.3">
@@ -76843,7 +77134,7 @@
       <c r="P33">
         <v>678967</v>
       </c>
-      <c r="Q33">
+      <c r="Q33" s="3">
         <v>678967</v>
       </c>
       <c r="R33" t="s">
@@ -76885,8 +77176,9 @@
       <c r="AD33">
         <v>678967</v>
       </c>
-      <c r="AE33" t="s">
-        <v>51</v>
+      <c r="AE33" t="e">
+        <f>VLOOKUP(Q33, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF33">
         <v>678967</v>
@@ -77275,9 +77567,9 @@
       <c r="FD33">
         <v>678967</v>
       </c>
-      <c r="FE33" t="str">
+      <c r="FE33" t="e">
         <f t="shared" si="0"/>
-        <v>J689123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="34" spans="1:161" x14ac:dyDescent="0.3">
@@ -77329,7 +77621,7 @@
       <c r="P34">
         <v>678967</v>
       </c>
-      <c r="Q34">
+      <c r="Q34" s="3">
         <v>678967</v>
       </c>
       <c r="R34" t="s">
@@ -77371,8 +77663,9 @@
       <c r="AD34">
         <v>678967</v>
       </c>
-      <c r="AE34" t="s">
-        <v>51</v>
+      <c r="AE34" t="e">
+        <f>VLOOKUP(Q34, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF34">
         <v>678967</v>
@@ -77761,9 +78054,9 @@
       <c r="FD34">
         <v>678967</v>
       </c>
-      <c r="FE34" t="str">
+      <c r="FE34" t="e">
         <f t="shared" si="0"/>
-        <v>J690123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="35" spans="1:161" x14ac:dyDescent="0.3">
@@ -77815,7 +78108,7 @@
       <c r="P35">
         <v>678967</v>
       </c>
-      <c r="Q35">
+      <c r="Q35" s="3">
         <v>678967</v>
       </c>
       <c r="R35" t="s">
@@ -77857,8 +78150,9 @@
       <c r="AD35">
         <v>678967</v>
       </c>
-      <c r="AE35" t="s">
-        <v>51</v>
+      <c r="AE35" t="e">
+        <f>VLOOKUP(Q35, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF35">
         <v>678967</v>
@@ -78247,9 +78541,9 @@
       <c r="FD35">
         <v>678967</v>
       </c>
-      <c r="FE35" t="str">
+      <c r="FE35" t="e">
         <f t="shared" si="0"/>
-        <v>J691123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="36" spans="1:161" x14ac:dyDescent="0.3">
@@ -78301,7 +78595,7 @@
       <c r="P36">
         <v>678967</v>
       </c>
-      <c r="Q36">
+      <c r="Q36" s="3">
         <v>678967</v>
       </c>
       <c r="R36" t="s">
@@ -78343,8 +78637,9 @@
       <c r="AD36">
         <v>678967</v>
       </c>
-      <c r="AE36" t="s">
-        <v>51</v>
+      <c r="AE36" t="e">
+        <f>VLOOKUP(Q36, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF36">
         <v>678967</v>
@@ -78733,9 +79028,9 @@
       <c r="FD36">
         <v>678967</v>
       </c>
-      <c r="FE36" t="str">
+      <c r="FE36" t="e">
         <f t="shared" si="0"/>
-        <v>J692123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="37" spans="1:161" x14ac:dyDescent="0.3">
@@ -78787,7 +79082,7 @@
       <c r="P37">
         <v>678967</v>
       </c>
-      <c r="Q37">
+      <c r="Q37" s="3">
         <v>678967</v>
       </c>
       <c r="R37" t="s">
@@ -78829,8 +79124,9 @@
       <c r="AD37">
         <v>678967</v>
       </c>
-      <c r="AE37" t="s">
-        <v>51</v>
+      <c r="AE37" t="e">
+        <f>VLOOKUP(Q37, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF37">
         <v>678967</v>
@@ -79219,9 +79515,9 @@
       <c r="FD37">
         <v>678967</v>
       </c>
-      <c r="FE37" t="str">
+      <c r="FE37" t="e">
         <f t="shared" si="0"/>
-        <v>J693123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="38" spans="1:161" x14ac:dyDescent="0.3">
@@ -79273,7 +79569,7 @@
       <c r="P38">
         <v>678967</v>
       </c>
-      <c r="Q38">
+      <c r="Q38" s="3">
         <v>678967</v>
       </c>
       <c r="R38" t="s">
@@ -79315,8 +79611,9 @@
       <c r="AD38">
         <v>678967</v>
       </c>
-      <c r="AE38" t="s">
-        <v>51</v>
+      <c r="AE38" t="e">
+        <f>VLOOKUP(Q38, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF38">
         <v>678967</v>
@@ -79705,9 +80002,9 @@
       <c r="FD38">
         <v>678967</v>
       </c>
-      <c r="FE38" t="str">
+      <c r="FE38" t="e">
         <f t="shared" si="0"/>
-        <v>J694123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="39" spans="1:161" x14ac:dyDescent="0.3">
@@ -79759,7 +80056,7 @@
       <c r="P39">
         <v>678967</v>
       </c>
-      <c r="Q39">
+      <c r="Q39" s="3">
         <v>678967</v>
       </c>
       <c r="R39" t="s">
@@ -79801,8 +80098,9 @@
       <c r="AD39">
         <v>678967</v>
       </c>
-      <c r="AE39" t="s">
-        <v>51</v>
+      <c r="AE39" t="e">
+        <f>VLOOKUP(Q39, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF39">
         <v>678967</v>
@@ -80191,9 +80489,9 @@
       <c r="FD39">
         <v>678967</v>
       </c>
-      <c r="FE39" t="str">
+      <c r="FE39" t="e">
         <f t="shared" si="0"/>
-        <v>J695123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="40" spans="1:161" x14ac:dyDescent="0.3">
@@ -80245,7 +80543,7 @@
       <c r="P40">
         <v>678967</v>
       </c>
-      <c r="Q40">
+      <c r="Q40" s="3">
         <v>678967</v>
       </c>
       <c r="R40" t="s">
@@ -80287,8 +80585,9 @@
       <c r="AD40">
         <v>678967</v>
       </c>
-      <c r="AE40" t="s">
-        <v>51</v>
+      <c r="AE40" t="e">
+        <f>VLOOKUP(Q40, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF40">
         <v>678967</v>
@@ -80677,9 +80976,9 @@
       <c r="FD40">
         <v>678967</v>
       </c>
-      <c r="FE40" t="str">
+      <c r="FE40" t="e">
         <f t="shared" si="0"/>
-        <v>J696123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="41" spans="1:161" x14ac:dyDescent="0.3">
@@ -80731,7 +81030,7 @@
       <c r="P41">
         <v>678967</v>
       </c>
-      <c r="Q41">
+      <c r="Q41" s="3">
         <v>678967</v>
       </c>
       <c r="R41" t="s">
@@ -80773,8 +81072,9 @@
       <c r="AD41">
         <v>678967</v>
       </c>
-      <c r="AE41" t="s">
-        <v>51</v>
+      <c r="AE41" t="e">
+        <f>VLOOKUP(Q41, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF41">
         <v>678967</v>
@@ -81163,9 +81463,9 @@
       <c r="FD41">
         <v>678967</v>
       </c>
-      <c r="FE41" t="str">
+      <c r="FE41" t="e">
         <f t="shared" si="0"/>
-        <v>J697123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="42" spans="1:161" x14ac:dyDescent="0.3">
@@ -81217,7 +81517,7 @@
       <c r="P42">
         <v>678967</v>
       </c>
-      <c r="Q42">
+      <c r="Q42" s="3">
         <v>678967</v>
       </c>
       <c r="R42" t="s">
@@ -81259,8 +81559,9 @@
       <c r="AD42">
         <v>678967</v>
       </c>
-      <c r="AE42" t="s">
-        <v>51</v>
+      <c r="AE42" t="e">
+        <f>VLOOKUP(Q42, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF42">
         <v>678967</v>
@@ -81649,9 +81950,9 @@
       <c r="FD42">
         <v>678967</v>
       </c>
-      <c r="FE42" t="str">
+      <c r="FE42" t="e">
         <f t="shared" si="0"/>
-        <v>J698123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="43" spans="1:161" x14ac:dyDescent="0.3">
@@ -81703,7 +82004,7 @@
       <c r="P43">
         <v>678967</v>
       </c>
-      <c r="Q43">
+      <c r="Q43" s="3">
         <v>678967</v>
       </c>
       <c r="R43" t="s">
@@ -81745,8 +82046,9 @@
       <c r="AD43">
         <v>678967</v>
       </c>
-      <c r="AE43" t="s">
-        <v>51</v>
+      <c r="AE43" t="e">
+        <f>VLOOKUP(Q43, Mapping!$D$2:$G$301,3,0)</f>
+        <v>#N/A</v>
       </c>
       <c r="AF43">
         <v>678967</v>
@@ -82135,9 +82437,9 @@
       <c r="FD43">
         <v>678967</v>
       </c>
-      <c r="FE43" t="str">
+      <c r="FE43" t="e">
         <f t="shared" si="0"/>
-        <v>J699123456789MMMM</v>
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>

</xml_diff>